<commit_message>
Updated files from NEXTGroup
</commit_message>
<xml_diff>
--- a/InputData/elec/BPMGBSA/BAU Policy Mandated Grid Battery Storage Additions.xlsx
+++ b/InputData/elec/BPMGBSA/BAU Policy Mandated Grid Battery Storage Additions.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\elec\BPMGBSA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kjh_local\04.AgentAI\02.EPS data updateAI\02.input_Korea\eps_4.0.5\elec\BPMGBSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{263E2315-08D3-4253-89E3-B080D235509A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03DB3C96-4699-41FD-94D0-BE06957DD67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="BPMGBSA" sheetId="2" r:id="rId2"/>
+    <sheet name="11차 전기본" sheetId="6" r:id="rId2"/>
+    <sheet name="BPMGBSA" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
   <si>
     <t>Source:</t>
   </si>
@@ -48,18 +49,58 @@
     <t>Capacity Additions</t>
   </si>
   <si>
-    <t>None</t>
+    <t>합계</t>
+  </si>
+  <si>
+    <t>https://www.motir.go.kr/kor/article/ATCLc01b2801b/70152/view</t>
+  </si>
+  <si>
+    <t>연도</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>필요물량(누적)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>신규설비(연도별)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>설비용량(누적)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>전국 (MW)</t>
+  </si>
+  <si>
+    <t>제주 (MW)</t>
+  </si>
+  <si>
+    <t>양수 (MW)</t>
+  </si>
+  <si>
+    <t>기타저장장치 (MW)</t>
+  </si>
+  <si>
+    <t>Ministry of Trade, Industry and Energy (MOTIE)</t>
+  </si>
+  <si>
+    <t>11th Basic Plan for Electricity Supply and Demand</t>
+  </si>
+  <si>
+    <t>10. Current Status and Plan for Energy Storage Systems (ESS)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -67,7 +108,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -75,20 +116,39 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDFE6F7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -96,12 +156,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -109,10 +184,29 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -125,6 +219,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>962744</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>124780</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="그림 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4EEAFA73-BEC0-2623-C436-DE79A97F1BEB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="5048250"/>
+          <a:ext cx="5153744" cy="6839905"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -412,197 +555,619 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="849" row="7">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{9C53C666-0ACB-4684-868E-8C90DFEFCD71}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B4" s="2"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B6" s="3"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B10" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0978A14-1A32-45AA-8A39-6995E772EF90}">
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="3" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="8">
+        <v>2023</v>
+      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="9">
+        <v>68</v>
+      </c>
+      <c r="F5" s="9">
+        <v>4700</v>
+      </c>
+      <c r="G5" s="8"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="8">
+        <v>2024</v>
+      </c>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="9">
+        <v>4700</v>
+      </c>
+      <c r="G6" s="8"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="8">
+        <v>2025</v>
+      </c>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="9">
+        <v>68</v>
+      </c>
+      <c r="F7" s="9">
+        <v>4700</v>
+      </c>
+      <c r="G7" s="8"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="8">
+        <v>2026</v>
+      </c>
+      <c r="B8" s="8"/>
+      <c r="C8" s="9">
+        <v>39</v>
+      </c>
+      <c r="D8" s="9">
+        <v>500</v>
+      </c>
+      <c r="E8" s="9">
+        <v>40</v>
+      </c>
+      <c r="F8" s="9">
+        <v>4700</v>
+      </c>
+      <c r="G8" s="9">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="8">
+        <v>2027</v>
+      </c>
+      <c r="B9" s="8"/>
+      <c r="C9" s="9">
+        <v>78</v>
+      </c>
+      <c r="D9" s="9">
+        <v>500</v>
+      </c>
+      <c r="E9" s="9">
+        <v>40</v>
+      </c>
+      <c r="F9" s="9">
+        <v>4700</v>
+      </c>
+      <c r="G9" s="9">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="8">
+        <v>2028</v>
+      </c>
+      <c r="B10" s="9">
+        <v>1000</v>
+      </c>
+      <c r="C10" s="9">
+        <v>117</v>
+      </c>
+      <c r="D10" s="9">
+        <v>500</v>
+      </c>
+      <c r="E10" s="9">
+        <v>40</v>
+      </c>
+      <c r="F10" s="9">
+        <v>4700</v>
+      </c>
+      <c r="G10" s="9">
+        <v>1688</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="8">
+        <v>2029</v>
+      </c>
+      <c r="B11" s="9">
+        <v>2100</v>
+      </c>
+      <c r="C11" s="9">
+        <v>155</v>
+      </c>
+      <c r="D11" s="9">
+        <v>600</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="9">
+        <v>4700</v>
+      </c>
+      <c r="G11" s="9">
+        <v>2288</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="8">
+        <v>2030</v>
+      </c>
+      <c r="B12" s="9">
+        <v>4000</v>
+      </c>
+      <c r="C12" s="9">
+        <v>194</v>
+      </c>
+      <c r="D12" s="9">
+        <v>500</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="9">
+        <v>5200</v>
+      </c>
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="8">
+        <v>2031</v>
+      </c>
+      <c r="B13" s="9">
+        <v>7600</v>
+      </c>
+      <c r="C13" s="9">
+        <v>233</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="9">
+        <v>5200</v>
+      </c>
+      <c r="G13" s="8"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="8">
+        <v>2032</v>
+      </c>
+      <c r="B14" s="9">
+        <v>10000</v>
+      </c>
+      <c r="C14" s="9">
+        <v>272</v>
+      </c>
+      <c r="D14" s="9">
+        <v>600</v>
+      </c>
+      <c r="E14" s="8"/>
+      <c r="F14" s="9">
+        <v>5800</v>
+      </c>
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="8">
+        <v>2033</v>
+      </c>
+      <c r="B15" s="9">
+        <v>12500</v>
+      </c>
+      <c r="C15" s="9">
+        <v>311</v>
+      </c>
+      <c r="D15" s="9">
+        <v>700</v>
+      </c>
+      <c r="E15" s="8"/>
+      <c r="F15" s="9">
+        <v>6500</v>
+      </c>
+      <c r="G15" s="8"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="8">
+        <v>2034</v>
+      </c>
+      <c r="B16" s="9">
+        <v>17500</v>
+      </c>
+      <c r="C16" s="9">
+        <v>350</v>
+      </c>
+      <c r="D16" s="9">
+        <v>1400</v>
+      </c>
+      <c r="E16" s="8"/>
+      <c r="F16" s="9">
+        <v>7900</v>
+      </c>
+      <c r="G16" s="8"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="8">
+        <v>2035</v>
+      </c>
+      <c r="B17" s="9">
+        <v>17500</v>
+      </c>
+      <c r="C17" s="9">
+        <v>388</v>
+      </c>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="9">
+        <v>7900</v>
+      </c>
+      <c r="G17" s="8"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="8">
+        <v>2036</v>
+      </c>
+      <c r="B18" s="9">
+        <v>20000</v>
+      </c>
+      <c r="C18" s="9">
+        <v>427</v>
+      </c>
+      <c r="D18" s="9">
+        <v>1500</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="F18" s="9">
+        <v>9400</v>
+      </c>
+      <c r="G18" s="8"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="8">
+        <v>2037</v>
+      </c>
+      <c r="B19" s="9">
+        <v>21000</v>
+      </c>
+      <c r="C19" s="9">
+        <v>466</v>
+      </c>
+      <c r="D19" s="9">
+        <v>1000</v>
+      </c>
+      <c r="E19" s="8"/>
+      <c r="F19" s="9">
+        <v>10400</v>
+      </c>
+      <c r="G19" s="8"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="8">
+        <v>2038</v>
+      </c>
+      <c r="B20" s="9">
+        <v>22500</v>
+      </c>
+      <c r="C20" s="9">
+        <v>505</v>
+      </c>
+      <c r="D20" s="9">
+        <v>1250</v>
+      </c>
+      <c r="E20" s="8"/>
+      <c r="F20" s="9">
+        <v>11650</v>
+      </c>
+      <c r="G20" s="8"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="11">
+        <v>9050</v>
+      </c>
+      <c r="E21" s="11">
+        <v>188</v>
+      </c>
+      <c r="F21" s="11">
+        <v>11650</v>
+      </c>
+      <c r="G21" s="11">
+        <v>2288</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AB2"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="6" width="8.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="C1">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="D1">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="E1">
-        <v>2023</v>
+        <v>2027</v>
       </c>
       <c r="F1">
-        <v>2024</v>
+        <v>2028</v>
       </c>
       <c r="G1">
-        <v>2025</v>
+        <v>2029</v>
       </c>
       <c r="H1">
-        <v>2026</v>
+        <v>2030</v>
       </c>
       <c r="I1">
-        <v>2027</v>
+        <v>2031</v>
       </c>
       <c r="J1">
-        <v>2028</v>
+        <v>2032</v>
       </c>
       <c r="K1">
-        <v>2029</v>
+        <v>2033</v>
       </c>
       <c r="L1">
-        <v>2030</v>
+        <v>2034</v>
       </c>
       <c r="M1">
-        <v>2031</v>
+        <v>2035</v>
       </c>
       <c r="N1">
-        <v>2032</v>
+        <v>2036</v>
       </c>
       <c r="O1">
-        <v>2033</v>
+        <v>2037</v>
       </c>
       <c r="P1">
-        <v>2034</v>
+        <v>2038</v>
       </c>
       <c r="Q1">
-        <v>2035</v>
+        <v>2039</v>
       </c>
       <c r="R1">
-        <v>2036</v>
+        <v>2040</v>
       </c>
       <c r="S1">
-        <v>2037</v>
+        <v>2041</v>
       </c>
       <c r="T1">
-        <v>2038</v>
+        <v>2042</v>
       </c>
       <c r="U1">
-        <v>2039</v>
+        <v>2043</v>
       </c>
       <c r="V1">
-        <v>2040</v>
+        <v>2044</v>
       </c>
       <c r="W1">
-        <v>2041</v>
+        <v>2045</v>
       </c>
       <c r="X1">
-        <v>2042</v>
+        <v>2046</v>
       </c>
       <c r="Y1">
-        <v>2043</v>
+        <v>2047</v>
       </c>
       <c r="Z1">
-        <v>2044</v>
+        <v>2048</v>
       </c>
       <c r="AA1">
-        <v>2045</v>
+        <v>2049</v>
       </c>
       <c r="AB1">
-        <v>2046</v>
-      </c>
-      <c r="AC1">
-        <v>2047</v>
-      </c>
-      <c r="AD1">
-        <v>2048</v>
-      </c>
-      <c r="AE1">
-        <v>2049</v>
-      </c>
-      <c r="AF1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="5">
+        <f>'11차 전기본'!$F$6</f>
+        <v>4700</v>
+      </c>
+      <c r="C2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,C$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,C$1)</f>
+        <v>68</v>
+      </c>
+      <c r="D2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,D$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,D$1)</f>
+        <v>540</v>
+      </c>
+      <c r="E2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,E$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,E$1)</f>
+        <v>540</v>
+      </c>
+      <c r="F2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,F$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,F$1)</f>
+        <v>540</v>
+      </c>
+      <c r="G2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,G$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,G$1)</f>
+        <v>600</v>
+      </c>
+      <c r="H2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,H$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,H$1)</f>
+        <v>500</v>
+      </c>
+      <c r="I2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,I$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,I$1)</f>
         <v>0</v>
       </c>
-      <c r="C2">
+      <c r="J2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,J$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,J$1)</f>
+        <v>600</v>
+      </c>
+      <c r="K2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,K$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,K$1)</f>
+        <v>700</v>
+      </c>
+      <c r="L2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,L$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,L$1)</f>
+        <v>1400</v>
+      </c>
+      <c r="M2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,M$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,M$1)</f>
         <v>0</v>
       </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
+      <c r="N2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,N$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,N$1)</f>
+        <v>1500</v>
+      </c>
+      <c r="O2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,O$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,O$1)</f>
+        <v>1000</v>
+      </c>
+      <c r="P2" s="5">
+        <f>SUMIFS('11차 전기본'!$D$5:$D$20,'11차 전기본'!$A$5:$A$20,P$1)+SUMIFS('11차 전기본'!$E$5:$E$20,'11차 전기본'!$A$5:$A$20,P$1)</f>
+        <v>1250</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -640,20 +1205,240 @@
       <c r="AB2">
         <v>0</v>
       </c>
-      <c r="AC2">
-        <v>0</v>
-      </c>
-      <c r="AD2">
-        <v>0</v>
-      </c>
-      <c r="AE2">
-        <v>0</v>
-      </c>
-      <c r="AF2">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="688c5d3b-a76a-458b-b159-91c2a1154680">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010027350D42B0D95040ACC873ED5DCB146E" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07e9ea90ad522b71e445466745b665d9">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="688c5d3b-a76a-458b-b159-91c2a1154680" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2528a4ec313a4f0a1f4e92f7a0496c8f" ns2:_="">
+    <xsd:import namespace="688c5d3b-a76a-458b-b159-91c2a1154680"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="688c5d3b-a76a-458b-b159-91c2a1154680" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="eca5b831-c3dc-41cf-bd85-218b82cecb21" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FDD2770E-9D51-43CB-AB57-4FB6607AE034}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="688c5d3b-a76a-458b-b159-91c2a1154680"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B496D2A-9A21-49CF-AC7C-EF74302CDBEF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6C54D5F-086A-4288-81B3-8CB9AD2A09D0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="688c5d3b-a76a-458b-b159-91c2a1154680"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>